<commit_message>
Add Rakuten review VOC (顧客の声) to research + refresh viewers
楽天/Yahoo!レビューの分析からVOC（顧客の声）を収集し、製品リサーチに追加。
テーマ別の良い声/気になる声と、ブログ活用マップを整理。

- libetee-product-research.xlsx：⑦顧客の声(VOC)、⑧レビュー活用マップ を追加(全8シート)
- HTML/PDF/Artifact(iPhone閲覧版)を再生成しVOCを反映
- 逐語引用を避け傾向を要約。出典明示・PR表記・デメリット併記の注意を明記

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UvmqjaSk6Q4EL44MiCWe3S
</commit_message>
<xml_diff>
--- a/suitcase-blog/libetee-product-research.xlsx
+++ b/suitcase-blog/libetee-product-research.xlsx
@@ -13,6 +13,8 @@
     <sheet name="④ 系統比較" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="⑤ ブログ対応表" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="⑥ 情報ソース" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="⑦ 顧客の声(VOC)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="⑧ レビュー活用マップ" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2682,4 +2684,591 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>顧客の声（VOC）｜楽天レビュー等の傾向</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>楽天/Yahoo!レビューを分析した各種調査記事より要約（調査日2026-08-04）。※原文の逐語引用ではなく傾向の要約。ブログ利用時は最新レビューを一次確認し、出典明示・PR表記・デメリット併記で中立に。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>テーマ</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>区分</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>声の要点（要約）</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>出典種別</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>ブログ／CVでの活かし方</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>静音性・キャスター</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>👍</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>HINOMOTO静音キャスターで走行音が静か・スムーズ。空港や住宅街でも快適（口コミ最評価点）</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>楽天</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>「静かさ」を検証記事/動画で実証。丈夫さ訴求と束ねる</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>フロントオープン</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>👍</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>立てたままPC/飲み物/お菓子をサッと取り出せて便利</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>楽天</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>出張・子連れ記事の主役機能に。実演写真を必須化</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>キャスターストッパー</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>👍</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>電車で手を離しても動かない。坂道・車内で安心</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Yahoo!/楽天</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>「キャスターロック」KW記事の実使用エピソードに</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>デザイン・高級感</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>👍</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>3万円台とは思えない高級感。さりげないロゴが好評</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>楽天</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>価格対価値の訴求。写真で質感を見せる</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>コスパ・多機能</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>👍</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>手頃な価格で機能が多い（ドリンクホルダー/USB/スマホスタンド）</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>楽天</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>比較記事の「機能×価格」軸で優位に</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>手入れ</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>👍</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>汚れが拭きやすい</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>口コミ</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>日常使い・清潔感の訴求に</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>耐久性</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>👍</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>頑丈で壊れにくく長く使える（永久保証も安心）</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>楽天</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>ボーケン試験＋永久保証と束ねTrust強化</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>重さ</t>
+        </is>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>⚠️</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>多機能ゆえ「少し重い」と感じる声</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>楽天/Yahoo!</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>実測重量を明記し「機能とのトレードオフ」を正直に説明</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>収納スペース</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>⚠️</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>フロントポケット分、内部容量がやや狭く感じる</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>口コミ</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>サイズ選びガイドで「多機能型は1サイズ上」も提案</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>初期不良</t>
+        </is>
+      </c>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>⚠️</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>キズ/ネジ落下/保護フィルムが剥がしにくい等の報告</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>楽天</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>永久保証・交換フローを明記し不安を先回りで解消</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>価格（上位）</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>⚠️</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>アルミ多機能など上位は「価格が高い」</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>口コミ</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>価格帯別おすすめで用途に合う型へ誘導</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>参考｜サイズ感：S 40L=2〜4泊(機内持込可) / M 65L=3〜7泊 / L 84L=7〜10泊</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>参考｜人気色：エナメルシルバー / マットブラック / マットホワイト</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>参考｜利用層：出張・子連れ・女性・修学旅行 など</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>⚠️ 逐語引用は避け傾向を要約。ブログ掲載時は最新レビューを一次確認し、出典（楽天/Yahoo!等）を明示。景表法/ステマ規制に留意しデメリットも併記。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A18:E18"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>レビュー活用マップ｜声をどの記事でどう使うか</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>VOCをE-E-A-T（実体験）・反論処理・比較の説得力に変換する。声はあくまで一次確認のうえ出典明示で使用。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>活用シーン</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>使う声（VOC）</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>対象商品／記事</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>具体アクション</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44" customHeight="1">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>E-E-A-T（実体験）</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>静音・フロントオープンの実使用感</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>全記事</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>著者の一次体験＋レビュー要約を併記（出典明示）</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>反論処理（重い）</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>「重い」の声</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>PC多機能／アルミ多機能</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>実測重量＋機能とのトレードオフを正直に。軽さ重視はジップ/クラシックへ誘導</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="44" customHeight="1">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>反論処理（初期不良）</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>初期不良の声</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>全商品</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>永久保証・交換フローを明記しCV前の不安を解消</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="44" customHeight="1">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>比較の説得力</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>コスパ・多機能の声</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>比較記事</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>「価格×機能」比較表の裏付けに引用</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="44" customHeight="1">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>キャスターロック記事</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>ストッパーの声</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>アルミ多機能／クラシック</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>電車・坂道の実使用エピソードで具体化</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="44" customHeight="1">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>サイズ選び</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>収納がやや狭いの声</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>サイズガイド</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>多機能型は1サイズ上を提案し満足度UP＆返品減</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>